<commit_message>
fix: standardize RIN field naming to lowercase 'rin' across the codebase
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/archiveExportTemplate.xlsx
+++ b/src/main/resources/templates/archiveExportTemplate.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ethan/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ethan/Mac本地文稿/0-本地项目/GezhiPlatform/src/main/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730F398E-66E4-2C40-9032-AF5DE824021F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E13A45E-5B2F-A145-856F-00056189EDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25660" yWindow="500" windowWidth="25540" windowHeight="26680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="学生信息登记表" sheetId="1" r:id="rId1"/>
@@ -208,10 +208,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>{RIN}</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>{juniorHighSchoolDistrict}</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -321,6 +317,10 @@
   </si>
   <si>
     <t>{mentalTreatment}</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>{rin}</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -514,86 +514,86 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,7 +864,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="40.5" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="29" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="19"/>
@@ -876,16 +876,16 @@
       <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="20" customHeight="1">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1">
       <c r="A3" s="18" t="s">
@@ -955,19 +955,19 @@
       <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="25"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="34"/>
       <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="24"/>
-      <c r="H6" s="25"/>
+      <c r="F6" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="33"/>
+      <c r="H6" s="34"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1">
       <c r="A7" s="18" t="s">
@@ -985,33 +985,33 @@
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="28"/>
+      <c r="B8" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="16"/>
+      <c r="D8" s="17"/>
       <c r="E8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="27"/>
-      <c r="H8" s="28"/>
+      <c r="F8" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="16"/>
+      <c r="H8" s="17"/>
     </row>
     <row r="9" spans="1:8" ht="18" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
+      <c r="B9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="1:8" ht="18" customHeight="1">
       <c r="A10" s="18" t="s">
@@ -1029,47 +1029,47 @@
       <c r="A11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
+      <c r="B11" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="32"/>
-      <c r="D12" s="33"/>
+      <c r="B12" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
       <c r="E12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="28"/>
+      <c r="F12" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
+      <c r="B13" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1">
       <c r="A14" s="18" t="s">
@@ -1101,55 +1101,55 @@
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="13"/>
-      <c r="D16" s="14"/>
+      <c r="B16" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="24"/>
+      <c r="D16" s="25"/>
       <c r="E16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="14"/>
+      <c r="F16" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="24"/>
+      <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
+      <c r="B17" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="27"/>
+      <c r="D17" s="28"/>
       <c r="E17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="17"/>
+      <c r="F17" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="27"/>
+      <c r="H17" s="28"/>
     </row>
     <row r="18" spans="1:8" ht="35" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
+      <c r="B18" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" s="24"/>
+      <c r="D18" s="25"/>
       <c r="E18" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="G18" s="13"/>
-      <c r="H18" s="14"/>
+      <c r="F18" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25"/>
     </row>
     <row r="19" spans="1:8" ht="16">
       <c r="A19" s="18" t="s">
@@ -1170,56 +1170,56 @@
         <v>4</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>28</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="35" customHeight="1">
       <c r="A21" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
+      <c r="B21" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="24"/>
+      <c r="D21" s="25"/>
       <c r="E21" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="G21" s="24"/>
+      <c r="H21" s="25"/>
+    </row>
+    <row r="22" spans="1:8" ht="18" customHeight="1">
+      <c r="A22" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="G21" s="13"/>
-      <c r="H21" s="14"/>
-    </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1">
-      <c r="A22" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="36"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="22"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1">
       <c r="A23" s="18" t="s">
@@ -1251,76 +1251,99 @@
       <c r="A25" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="14"/>
+      <c r="B25" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
       <c r="E25" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="G25" s="13"/>
-      <c r="H25" s="14"/>
+      <c r="F25" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="G25" s="24"/>
+      <c r="H25" s="25"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1">
       <c r="A26" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C26" s="16"/>
-      <c r="D26" s="17"/>
+      <c r="B26" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="27"/>
+      <c r="D26" s="28"/>
       <c r="E26" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="G26" s="16"/>
-      <c r="H26" s="17"/>
+      <c r="F26" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" s="27"/>
+      <c r="H26" s="28"/>
     </row>
     <row r="27" spans="1:8" ht="60" customHeight="1">
       <c r="A27" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="12"/>
+      <c r="B27" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="35"/>
+      <c r="D27" s="36"/>
       <c r="E27" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G27" s="11"/>
-      <c r="H27" s="12"/>
+      <c r="F27" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
     </row>
     <row r="28" spans="1:8" ht="60" customHeight="1">
       <c r="A28" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="12"/>
+      <c r="B28" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="35"/>
+      <c r="D28" s="36"/>
       <c r="E28" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="12"/>
+      <c r="F28" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="G28" s="35"/>
+      <c r="H28" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="A10:H10"/>
     <mergeCell ref="B11:H11"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B12:D12"/>
@@ -1337,29 +1360,6 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="B9:H9"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="F26:H26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="F27:H27"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>